<commit_message>
Syllabus and schedule follow the data plan
Labs 1-7 run in the Houtan Coffee world and Labs 8-9 on Airbnb; A1-A2 use Hillstrom (A2 retitled for
email), A3 uses dunnhumby with a locked simulator (no LLM-coded feature), A4 uses Favorita. Assignments
are graded on the pipeline, not a score. Objective 3 covers pricing. FLAGS line references follow the
syllabus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -536,7 +536,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1086,11 +1085,10 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Labs 1 to 11 go with Meetings 1 to 11. Ten are graded, 1 point each; Lab 7 is optional and ungraded (its methods are graded in A3). Notebooks are expected soon after their meeting. AI roles: tool (Lab 2), decision-maker (Lab 5), analyst (Lab 7, optional), source of data (Lab 9), intervention (Lab 10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
+          <t>Labs 1 to 11 go with Meetings 1 to 11. Ten are graded, 1 point each; Lab 7 is optional and ungraded (its methods are graded in A3). Notebooks are expected soon after their meeting. AI roles: tool (Lab 2), decision-maker (Lab 5), analyst (Lab 7, optional), source of data (Lab 9), intervention (Lab 10). Each block of labs works in one semi-synthetic world with a planted truth: Labs 1 to 7 in Houtan Coffee's loyalty program (built on the Starbucks rewards data from Kaggle), Labs 8 and 9 in Airbnb listings and reviews (Inside Airbnb; the city is chosen later), Labs 10 and 11 in real store panels with planted rollouts. Notebooks describe their source data.</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1126,12 +1124,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Review; simulation from scratch</t>
+          <t>Review; semi-synthetic</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Simulated</t>
+          <t>Houtan Coffee world, simulated from scratch</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1153,12 +1151,12 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Real data and simulation; LLM lab</t>
+          <t>Semi-synthetic; LLM lab</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Email experiment (Hillstrom)</t>
+          <t>Houtan Coffee RCT (randomization, effects and pre-period spend planted)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -1180,12 +1178,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>From scratch; simulation</t>
+          <t>Semi-synthetic</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Three simulated worlds with known CATE (no heterogeneity, strong heterogeneity, 10% treated)</t>
+          <t>Houtan Coffee RCT, three versions with different planted CATE (no heterogeneity, strong heterogeneity, 10% treated)</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1207,12 +1205,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Real data</t>
+          <t>Semi-synthetic</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Coupon RCT</t>
+          <t>Houtan Coffee RCT</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1234,12 +1232,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Real data; LLM lab</t>
+          <t>Semi-synthetic; LLM lab</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Coupon RCT holdout, with text profiles generated from the features</t>
+          <t>Houtan Coffee RCT holdout, with text profiles generated from the features</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1261,12 +1259,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>From scratch (optimization); real data</t>
+          <t>From scratch (optimization); semi-synthetic</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Coupon RCT with customer-specific costs and three coupon depths</t>
+          <t>Houtan Coffee RCT with customer-specific costs and three coupon depths</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1293,7 +1291,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Logs built from the coupon RCT by a known targeting rule, with a post-treatment variable and a collider among the columns</t>
+          <t>Logs built from the Houtan Coffee RCT by a known targeting rule (overlap dial), with a post-treatment variable and a collider among the columns; truth from the RCT version</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1315,12 +1313,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Real data; from scratch (in class)</t>
+          <t>Semi-synthetic on real listings; from scratch (in class)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Orange-juice scanner data (Dominick's)</t>
+          <t>Airbnb listings and host prices; demand with a planted heterogeneous elasticity, confounded by a latent quality carried in the review text</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -1330,7 +1328,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Naive, fixed-effects and DML elasticities; hand-code partialling-out with cross-fitting, then match DoubleML; stability across learners and splits; sensitivity bounds (how much hidden confounding flips the pricing decision)</t>
+          <t>Naive, fixed-effects and DML elasticities; hand-code partialling-out with cross-fitting, then match DoubleML; stability across learners and splits; the optimal price; sensitivity bounds (how much hidden confounding flips the pricing decision)</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1345,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Public hotel reviews; treatment and bookings simulated from a quality variable carried in the text; gold labels on a subsample</t>
+          <t>Airbnb reviews; the latent quality is planted, with gold labels on a subsample</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1357,7 +1355,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Compare LLM labels with gold, including error by treatment arm; use the label as an outcome with and without PPI; embeddings as DML controls vs the truth; a leakage demo with post-treatment text</t>
+          <t>Compare LLM labels with gold quality, including error by treatment arm; use the label as an outcome with and without PPI; embeddings as DML controls vs the truth; a leakage demo with post-treatment text; a simulator with a confounding dial</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1496,7 +1494,7 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>On a second email campaign: hand-code the ATE with a robust SE, and CUPED. Have an LLM generate the full readout (SRM, ATE, CUPED, test against the break-even, MDE for a follow-up) and verify it with a simulation test suite. One-page decision memo</t>
+          <t>On the Hillstrom email RCT (resampled, with course-specific costs): hand-code the ATE with a robust SE, and CUPED on history. Have an LLM generate the full readout (SRM, ATE, CUPED, test against the break-even, MDE for a follow-up) and verify it with a simulation test suite. One-page decision memo</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1508,7 +1506,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>A2: Coupon whom, and at what budget?</t>
+          <t>A2: Email whom, and at what budget?</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -1528,7 +1526,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>CATE from two meta-learners and a causal forest; ranking evaluated with Qini and RATE; a budgeted allocation and a depth-2 policy tree. Frozen policies are submitted and scored by an autograder on a locked RCT set. Memo on value, cost, and what could overturn the recommendation</t>
+          <t>Hillstrom, three arms (men's email, women's email, no email). CATE from two meta-learners and a causal forest; ranking evaluated with Qini and RATE; a budgeted allocation and a depth-2 policy tree. Frozen policies are scored by IPW on a locked holdout of at least 20,000 rows, with paired comparisons. Memo on value, cost, and what could overturn the recommendation</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -1540,7 +1538,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>A3: Learn the policy from the logs</t>
+          <t>A3: Promote and price from the logs</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -1560,7 +1558,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>The same decision, from observational logs only. (1) DAG and adjustment set; regression, IPW and AIPW estimates; overlap and trimming (the methods of Lab 7). (2) DML on the same logs, compared with (1) and with the locked RCT. (3) Generative AI for evaluation: a simulator fitted to the coupon logs, with a planted effect and a dial for hidden confounding, as a testbed for each estimator's bias and coverage and for whether the policy ranking holds as confounding grows. An LLM-coded feature is to be decided (depends on the problem and data). The submitted policy is scored on the locked RCT set next to an RCT-trained benchmark. Memo with a sensitivity bound: how strong hidden confounding must be to change the chosen policy</t>
+          <t>dunnhumby "Breakfast at the Frat" (real grocery data, no experiment). (1) The effect of an in-store display: DAG and adjustment set; regression, IPW and AIPW estimates; overlap and trimming (the methods of Lab 7). (2) The price elasticity by DML, and a recommended price. (3) Generative AI for evaluation: a student-built simulator of the data with a planted elasticity and a dial for hidden confounding, as a testbed for each estimator's bias and coverage. The pipeline is then run on the instructor's locked simulator across several planted-elasticity scenarios. Memo with a sensitivity bound: how strong hidden confounding must be to change the recommended price</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1592,12 +1590,19 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Panel data. Evaluate the rollout of an AI store assistant: before-after, 2x2 DiD and TWFE with store and period effects; an event study; what the pre-period can and cannot rule out (breakdown drift); store-clustered SEs; why staggered timing needs a different design. Then a synthetic control for one flagship store, with placebos and leave-one-out, and a comparison with DiD. Decision memo in margin, not sales</t>
+          <t>Favorita grocery panel with a planted rollout of an AI store assistant, adoption tied to the stores' real pre-trends; the April 2016 earthquake falls in the window. Before-after, 2x2 DiD and TWFE with store and period effects; an event study; what the pre-period can and cannot rule out (breakdown drift); store-clustered SEs; a small second wave and why staggered timing needs a different design. Then a synthetic control for one flagship store, with placebos and leave-one-out, and a comparison with DiD. Decision memo in margin, not sales</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Allowed, disclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Assignments use real data that no lab touches. Each is graded on a complete, well-reasoned analysis pipeline, not on a performance score.</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1634,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1822,7 +1826,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -2151,12 +2154,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>A2 and A3 ask the same question</t>
+          <t>A2 and A3 use different data</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Logs-trained policy scored next to the RCT-trained one on a locked evaluation set; needs an autograder.</t>
+          <t>Decided (10 Oct): A2 scores frozen policies on a locked Hillstrom holdout; A3 uses dunnhumby and is scored on a locked simulator. The RCT-versus-logs comparison on one locked set is dropped. The LLM-coded feature is in Lab 9, not A3.</t>
         </is>
       </c>
     </row>
@@ -2224,7 +2227,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Lab 9 (cached LLM outputs, gold labels) and the A3 simulator of the coupon logs (built on the generator behind Lab 7) need the most up-front work.</t>
+          <t>The Houtan Coffee world (Labs 1 to 7, from 20 Oct), the Hillstrom file (A1, 22 Oct), Lab 9 (cached LLM outputs, gold labels), and the A3 locked simulator need the most up-front work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Schedule: observational methods before policy learning; blocks redistributed
Instructor's restructure: trees and forests in one block with CATE evaluation in M4; allocation in M5B;
observational data in M6 and DML in M7, so propensity scores and double robustness come before policy
learning, which moves to M8B after the proposal presentations. Lecture blocks keep the concepts;
mechanics (peeking, variable importance, isotonic recalibration, coupon depths, repeated splits,
choice of learners) move into the labs. Shading, releases, bonus reading and handouts follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DLgfSPmYNxNjqrXY4qwk61
</commit_message>
<xml_diff>
--- a/plan/schedule.xlsx
+++ b/plan/schedule.xlsx
@@ -536,7 +536,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -605,7 +604,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Lab 1: Python, probability and statistics review</t>
+          <t>Lab 1: Python, probability and statistics review; a potential-outcomes simulator that checks naive difference = ATT + selection bias</t>
         </is>
       </c>
       <c r="F4" s="4" t="n"/>
@@ -633,12 +632,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Experiments II: design. Fixing the plan in writing; power and MDE for a decision; CUPED; randomization unit, interference and clustered SEs; peeking and multiple metrics; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
+          <t>Experiments II: design. Fixing the plan in writing; power and MDE for a decision; CUPED; randomization unit, interference and clustered SEs; to close, noncompliance in an RCT: ITT and first stage, compliance types, the LATE (potential outcomes; the draw as the instrument)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Lab 2: A/B readout, then an LLM-generated readout checked by simulation tests</t>
+          <t>Lab 2: A/B readout by hand (SRM, robust SE, CUPED, test against the break-even); then an LLM-generated readout checked by simulation tests (planted-effect coverage, size under the null, the cost of peeking, multiple metrics)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -678,12 +677,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>CATE II: models. S-, T-, X-learners; transformed outcome; DR- and R-learners; TARNet as a shared representation; choosing a model without ground truth (R-loss, DR pseudo-outcomes)</t>
+          <t>CATE II: models. S-, T-, X-learners; transformed outcome; DR- and R-learners with the known propensity of an RCT (double robustness waits for M6); TARNet as a shared representation; choosing a model without ground truth (R-loss, pseudo-outcomes)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Lab 3: meta-learners from scratch</t>
+          <t>Lab 3: meta-learners from scratch on three Houtan Coffee worlds with different planted effects; a provided TARNet notebook</t>
         </is>
       </c>
       <c r="F6" s="4" t="n"/>
@@ -714,20 +713,24 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>CATE III: causal trees. An estimand chosen by the data; causal trees that split on effect heterogeneity; the winner's curse; honesty and sample splitting; committing a discovery (discover, estimate, recommend)</t>
+          <t>CATE III: causal trees and forests. An estimand chosen by the data; causal trees that split on effect heterogeneity; the winner's curse; honesty and sample splitting; committing a discovery (discover, estimate, recommend); forests as adaptive neighbors and the forest estimate (link to the R-learner); CATE intervals and their limits</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>CATE IV: causal forests. Forests as adaptive neighbors; the forest estimate and local centering (link to the R-learner); CATE intervals and their limits; variable-importance pitfalls; BLP calibration test and GATES</t>
+          <t>CATE IV: evaluation. Testing for heterogeneity on held-out data (BLP calibration test, GATES); policy value and the policy-value identity; IPW value with the known propensity, and its variance; gain, profit and Qini curves; RATE; ranking vs calibration; selection vs evaluation data and freezing a policy; comparing two policies (paired SE)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Lab 4: causal forest on the coupon RCT</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
+          <t>Lab 4: causal forest with and without honesty across seeds; variable importance vs the calibration test; four targeting rules (one chosen by an LLM reading profiles) evaluated by IPW, Qini and RATE; isotonic recalibration</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
           <t>A1 (Fri 30 Oct)</t>
@@ -735,7 +738,7 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>Forest theory</t>
+          <t>Forest theory; evaluating prioritization rules</t>
         </is>
       </c>
       <c r="I7" s="6" t="n"/>
@@ -756,29 +759,21 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>CATE V: evaluation. Policy value and the policy-value identity; IPW value on held-out RCT data and its variance; gain, profit and Qini curves; RATE; ranking vs calibration, and isotonic recalibration; selection vs evaluation data; freezing a policy; comparing two policies (paired SE)</t>
+          <t>CATE V: allocation and decision. Net value per customer and break-even thresholds; customer-specific costs and the sure-thing cost; contact caps; budget as a knapsack and its shadow price; group constraints and the price of fairness; spending risk, noisy estimates and lower-bound allocation; capacity and the critical fractile; what the sum assumes (interference, support)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Lab 5: CATE evaluation: four targeting rules (one chosen by an LLM) by IPW, Qini and RATE, isotonic recalibration, freeze then evaluate, paired comparison</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
+          <t>Lab 5: CATE allocation: greedy and LP allocation under a budget and caps; the shadow price; several coupon depths; lower-bound allocation; the price of a group constraint; allocations compared on held-out value with a paired comparison</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="n"/>
       <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Proposal (Sun 8 Nov)</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Evaluating prioritization rules</t>
-        </is>
-      </c>
+      <c r="H8" s="8" t="n"/>
       <c r="I8" s="8" t="n"/>
     </row>
     <row r="9">
@@ -792,111 +787,111 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>CATE VI: allocation. Net value per customer and break-even thresholds; customer-specific costs and the sure-thing cost; contact caps; budget as a knapsack and its shadow price; several coupon depths; group constraints and the price of fairness; spending risk and the reserve; noisy estimates and lower-bound allocation; capacity and the critical fractile</t>
+          <t>Observational data I: identification and adjustment. Logs produced by a targeting rule; exchangeability, overlap, consistency; standardization (g-computation) and IPW with an estimated propensity; the balancing property; what regression adjustment estimates; good and bad controls (mediators, colliders, M-bias, post-treatment variables)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>CATE VII: policy learning. Predict-then-optimize, decision-focused learning and policy learning as one spectrum; empirical welfare maximization with DR scores; policy learning as weighted classification; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation; what the sum assumes (interference, support)</t>
+          <t>Observational data II: overlap, design and double robustness. Overlap diagnostics, trimming and the changed estimand; the outcome-free design stage; doubly robust AIPW (and why the M3 DR-learner works); the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Lab 6: budgeted allocation and policy trees</t>
+          <t>Lab 6: observational data: logs built from the Houtan Coffee RCT by a known targeting rule; DAG and adjustment set; naive, regression, IPW, AIPW and matching against the RCT truth; overlap and trimming; then audit a tool-calling agent's analysis and add a guardrail</t>
         </is>
       </c>
       <c r="F9" s="6" t="n"/>
       <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="inlineStr">
         <is>
+          <t>Instrumental variables</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>H4 Instrumental variables</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Tue 10 Nov</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>DML I. The partially linear model; residualization (FWL) and what theta averages when effects vary; why plug-in ML fails (regularization and overfitting bias); cross-fitting; orthogonality in words; price elasticity</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DML II. Overlap with a continuous treatment; the interactive model and AIPW scores; DML for CATE; inference with cross-fitting; omitted-variable sensitivity bounds and benchmarking</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Lab 7: DML from scratch on Airbnb listings: naive, fixed-effects and DML elasticities; hand-coded cross-fitting, then match a package; stability across nuisance learners and repeated splits; sensitivity bounds; the optimal price</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Regression discontinuity</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>H5 Regression discontinuity</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Thu 12 Nov</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>PROPOSAL PRESENTATIONS</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Policy learning from observational data. Predict-then-optimize, decision-focused learning and policy learning as one spectrum; cross-fitted DR scores from logs; empirical welfare maximization; policy learning as weighted classification; policy trees; regret and policy-class complexity; deploying with holdouts; bandits as continuous experimentation</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>Lab 8: policy learning from the Houtan Coffee logs: cross-fitted DR scores; a depth-2 policy tree vs plug-in targeting; both evaluated on the RCT holdout</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>A2 (Sun 15 Nov)</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
           <t>Policy learning theory; dynamic regimes</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>H3 Sequential decisions</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Tue 10 Nov</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Observational data I: identification and adjustment. Logs produced by a targeting rule; exchangeability, overlap, consistency; standardization (g-computation) and IPW; the balancing property; what regression adjustment estimates; good and bad controls (mediators, colliders, M-bias, post-treatment variables)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Observational data II: overlap, design and double robustness. Overlap diagnostics, trimming and the changed estimand; the outcome-free design stage; doubly robust AIPW; the LaLonde benchmark; a first look at sensitivity to hidden confounding</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>PROPOSAL PRESENTATIONS. Lab 7 (optional, ungraded, take-home): observational methods on logs built from an RCT, then an agent's analysis audited</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>A3</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Instrumental variables</t>
-        </is>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>H4 Instrumental variables</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Thu 12 Nov</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>DML I. The partially linear model; residualization (FWL) and what theta averages when effects vary; why plug-in ML fails (regularization and overfitting bias); cross-fitting; orthogonality in words; price elasticity</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>DML II. Inference and repeated splits; choice of nuisance learners; overlap with a continuous treatment; the interactive model and AIPW scores; DML for CATE; omitted-variable sensitivity bounds and benchmarking</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Lab 8: DML on Airbnb listings (in class)</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>A2 (Sun 15 Nov)</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Regression discontinuity</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>H5 Regression discontinuity</t>
         </is>
       </c>
     </row>

</xml_diff>